<commit_message>
Update Paper count all Stages 19.12.2025.xlsx
</commit_message>
<xml_diff>
--- a/01_Search_Strategy/Paper count all Stages 19.12.2025.xlsx
+++ b/01_Search_Strategy/Paper count all Stages 19.12.2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rao\Documents\Towards PHD Cyber Security and CNI\Proposals\Journal Submition paper\SLR 2026\SLR-Insider-Threat-Detection-ML-Supplement Alriyami Murtadha - Final Copy\01_Search_Strategy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rao\Documents\Towards PHD Cyber Security and CNI\Proposals\Journal Submition paper\SLR 2026\PLOS One\SLR-Insider-Threat-Detection-ML-Supplement Alriyami Murtadha - Final Copy\01_Search_Strategy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF356994-0F50-4F86-9902-5492CE1FD045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FCC14AA-DDB2-4CCE-8505-F3E5C514F263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C5027576-2AE3-42F9-9AD9-DD288F20F753}"/>
   </bookViews>
@@ -84,7 +84,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -123,6 +123,28 @@
     <font>
       <b/>
       <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -155,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -174,12 +196,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -521,10 +545,10 @@
     <col min="4" max="4" width="22.83203125" customWidth="1"/>
     <col min="5" max="5" width="19.83203125" customWidth="1"/>
     <col min="6" max="6" width="17.58203125" customWidth="1"/>
-    <col min="7" max="7" width="27" customWidth="1"/>
+    <col min="7" max="7" width="27.58203125" customWidth="1"/>
     <col min="8" max="8" width="42.08203125" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="27" customWidth="1"/>
-    <col min="10" max="10" width="21.6640625" customWidth="1"/>
+    <col min="9" max="9" width="33.58203125" customWidth="1"/>
+    <col min="10" max="10" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="3:10" ht="18" x14ac:dyDescent="0.4">
@@ -535,28 +559,28 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="3:10" ht="18" x14ac:dyDescent="0.4">
+    <row r="9" spans="3:10" ht="20" x14ac:dyDescent="0.4">
       <c r="C9" s="1"/>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="1" t="s">
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="3:10" ht="24.5" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="9" t="s">
         <v>0</v>
       </c>
       <c r="D10" s="3">
@@ -582,7 +606,7 @@
       </c>
     </row>
     <row r="11" spans="3:10" ht="31" x14ac:dyDescent="0.7">
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D11" s="3">
@@ -608,7 +632,7 @@
       </c>
     </row>
     <row r="12" spans="3:10" ht="31" x14ac:dyDescent="0.7">
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="9" t="s">
         <v>5</v>
       </c>
       <c r="D12" s="3">
@@ -634,7 +658,7 @@
       </c>
     </row>
     <row r="13" spans="3:10" ht="31" x14ac:dyDescent="0.7">
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="3">
@@ -660,7 +684,7 @@
       </c>
     </row>
     <row r="14" spans="3:10" ht="31" x14ac:dyDescent="0.7">
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="3">
@@ -685,8 +709,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="3:10" ht="18" x14ac:dyDescent="0.4">
-      <c r="C15" s="1"/>
+    <row r="15" spans="3:10" ht="20" x14ac:dyDescent="0.4">
+      <c r="C15" s="9"/>
       <c r="D15" s="4">
         <f>SUM(D10:D14)</f>
         <v>1949</v>
@@ -716,8 +740,8 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="3:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C16" s="1" t="s">
+    <row r="16" spans="3:10" ht="20" x14ac:dyDescent="0.4">
+      <c r="C16" s="9" t="s">
         <v>2</v>
       </c>
       <c r="D16" s="2">
@@ -743,26 +767,17 @@
       </c>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="D17" s="9">
+    <row r="17" spans="3:8" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="D17" s="8">
         <f>D16+E16</f>
         <v>1286</v>
       </c>
-      <c r="E17" s="9"/>
+      <c r="E17" s="8"/>
       <c r="H17" s="7"/>
     </row>
     <row r="20" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="G20">
-        <v>124</v>
-      </c>
       <c r="H20" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="21" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="G21">
-        <f>G20/2</f>
-        <v>62</v>
       </c>
     </row>
     <row r="24" spans="3:8" x14ac:dyDescent="0.3">

</xml_diff>